<commit_message>
Revisão final: correções da seção 4.15 (carga interna) e reconciliações
- PSE final (Tab. 46/47/53): corrigido de 8,5/8,5/9,1 para 9,3/9,3/9,6 (média da
  última série); Friedman do PSE entre sessões corrigido para n.s. (p=0,45).
- Confirmado que Tab. 25 (por observação) e Tab. 48/55 (por dia, 2 passos) reproduzem
  exatamente — mesma comparação sob ponderações diferentes; notas de legenda acrescentadas.
- Deriva cardíaca esclarecida (subida total entre séries) na legenda.
- Apêndice B, relatório, workbook e CSV de verificação atualizados (84 checagens; 77 OK).
- Carga interna FC/PSE (FC de pico, ICC, deriva) reproduzida a partir dos dados brutos.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0157sZ1CmW4MRSmx6a9GoYrN
</commit_message>
<xml_diff>
--- a/auditoria_brums_hiit/Auditoria_BRUMS_HIIT.xlsx
+++ b/auditoria_brums_hiit/Auditoria_BRUMS_HIIT.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -584,50 +584,71 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2) Pequenas divergências a reconciliar (não alteram conclusões):</t>
+          <t xml:space="preserve">  2) Correções/reconciliações aplicadas ao manuscrito (Apêndice B):</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">     - Resposta aguda: dz recalculado (fadiga física 0,76) coincide com o RESUMO, não com a Tab.22 (0,71).</t>
+          <t xml:space="preserve">     - Resposta aguda (Tab.22): dz adotado = recalculado (fadiga física 0,76), coerente com o Resumo.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">     - Tab.2: "% piso" do PTH (21,9) não é reproduzível (PTH não tem piso em 0).</t>
+          <t xml:space="preserve">     - Tab.2: "% piso" do PTH (21,9) -&gt; "—" (PTH não tem piso em 0).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">     - PSE final (Tab.46): recalculado ~9,4 na última série vs 8,5 reportado — checar definição.</t>
+          <t xml:space="preserve">     - Carga interna: PSE final corrigido para 9,3/9,3/9,6 (última série); Friedman do PSE n.s. (p=0,45).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3) CFA (WLSMV ordinal), TRI/GRM, HTMT policórico e invariância exigem R (lavaan/mirt/semTools);</t>
+          <t xml:space="preserve">     - Referência duplicada removida; notas de agregação (Tab.25 x 48) e deriva cardíaca acrescentadas.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">     não foram reexecutados em Python — recomenda-se replicação de script.</t>
+          <t xml:space="preserve">  3) Confirmado que Tab.25 (por observação) e Tab.48/55 (por dia, 2 passos) reproduzem exatamente:</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     são a mesma comparação sob ponderações diferentes; ambas convergem.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4) CFA (WLSMV ordinal), TRI/GRM, HTMT policórico, invariância e BF bayesiano exigem R (lavaan/mirt/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     semTools/BayesFactor) — não reexecutados em Python; recomenda-se replicação de script.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>Atletas anonimizados (A01–A27). O mapa de códigos pode diferir do usado no artigo.</t>
         </is>
@@ -644,7 +665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E79"/>
+  <dimension ref="A1:E85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2241,7 +2262,7 @@
       </c>
       <c r="E69" s="6" t="inlineStr">
         <is>
-          <t>≈ (resumo usa 0,76 p/ fadiga física)</t>
+          <t>RECONCILIADO (adotado o dz recalculado; ver Apêndice B)</t>
         </is>
       </c>
     </row>
@@ -2264,7 +2285,7 @@
       </c>
       <c r="E70" s="6" t="inlineStr">
         <is>
-          <t>≈ (resumo usa 0,76 p/ fadiga física)</t>
+          <t>RECONCILIADO (adotado o dz recalculado; ver Apêndice B)</t>
         </is>
       </c>
     </row>
@@ -2287,7 +2308,7 @@
       </c>
       <c r="E71" s="6" t="inlineStr">
         <is>
-          <t>≈ (resumo usa 0,76 p/ fadiga física)</t>
+          <t>RECONCILIADO (adotado o dz recalculado; ver Apêndice B)</t>
         </is>
       </c>
     </row>
@@ -2310,7 +2331,7 @@
       </c>
       <c r="E72" s="6" t="inlineStr">
         <is>
-          <t>≈ (resumo usa 0,76 p/ fadiga física)</t>
+          <t>RECONCILIADO (adotado o dz recalculado; ver Apêndice B)</t>
         </is>
       </c>
     </row>
@@ -2467,11 +2488,149 @@
         <v>8.5</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>9.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>DIVERGE (última série ~9,4)</t>
+          <t>CORRIGIDO → 9,3/9,3/9,6 (última série); Friedman n.s. (p=0,45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>Tab.48 HIIT (2 passos) dz</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Vigor</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="n">
+        <v>-0.67</v>
+      </c>
+      <c r="D80" s="4" t="n">
+        <v>-0.67</v>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>Tab.48 HIIT (2 passos) dz</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>PTH</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D81" s="4" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="E81" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>Tab.48 HIIT (2 passos) dz</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>Fadiga</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="D82" s="4" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>Tab.48 HIIT (2 passos) dz</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>FadFis</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="D83" s="4" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>Tab.47 Carga interna</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>FC pico ICC(1,1)</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="D84" s="4" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="E84" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>Tab.53 Carga interna</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>PSE Friedman (entre sessões)</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="D85" s="4" t="n">
+        <v>0.447</v>
+      </c>
+      <c r="E85" s="6" t="inlineStr">
+        <is>
+          <t>CORRIGIDO (n.s.)</t>
         </is>
       </c>
     </row>

</xml_diff>